<commit_message>
changed the test files
</commit_message>
<xml_diff>
--- a/tests/fixtures/sample.xlsx
+++ b/tests/fixtures/sample.xlsx
@@ -7,8 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legacy" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unicode" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="සංචාරක ස්ථාන" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,27 +26,37 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="FMAbhaya"/>
-    </font>
-    <font>
-      <name val="FMBindumathix"/>
-    </font>
-    <font>
-      <name val="Nirmala UI"/>
+      <name val="Iskoola Pota"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Iskoola Pota"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+        <bgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -55,16 +64,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00DDDDDD"/>
+      </left>
+      <right style="thin">
+        <color rgb="00DDDDDD"/>
+      </right>
+      <top style="thin">
+        <color rgb="00DDDDDD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00DDDDDD"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,62 +458,254 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="65" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>wOHdmk m%ldYk fomd¾;fïka;=j</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>www.edupub.gov.lk</t>
+          <t>සංචාරක ස්ථානය</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>දිස්ත්‍රික්කය</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>වටිනාකම / ප්‍රවේශ ගාස්තුව</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>විස්තරය</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>wOHdmk m%ldYk fomd¾;fïka;=j</t>
+          <t>සීගිරිය</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>මාතලේ</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>රු. 100 (දේශීය)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>පැරණි බලකොටුව සහ ලෝක ප්‍රකට බිතුසිතුවම් සහිත යුනෙස්කෝ උරුමයකි.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" t="n">
-        <v>42</v>
-      </c>
-      <c r="C3">
-        <f>B3*2</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>අධ්‍යාපන ප්‍රකාශන දෙපාර්තමේන්තුව</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>සියලු ම පෙළපොත් නොමිලේ බෙදා දෙනු ලැබේ</t>
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>ශ්‍රී දළදා මාළිගාව</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>මහනුවර</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>නොමිලේ (දේශීය)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>බුදුරජාණන් වහන්සේගේ වාම ශ්‍රී දළදාව තැන්පත් කර ඇති පූජනීය ස්ථානයයි.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>ගාලු කොටුව</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>ගාල්ල</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>නොමිලේ</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>පෘතුගීසි සහ ලන්දේසි යුගයේ ඉදිකළ, යුනෙස්කෝ ලෝක උරුමයක් වන ඓතිහාසික බලකොටුවකි.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>යාල ජාතික වනෝද්‍යානය</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>හම්බන්තොට</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>රු. 150 (දේශීය)</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>දිවියන්, අලි ඇතුන් සහ විවිධ වන සතුන් නැරඹීම සඳහා ප්‍රසිද්ධතම වනෝද්‍යානයයි.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>ඇල්ල</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>බදුල්ල</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>නොමිලේ</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>සොබාදහමේ සුන්දරත්වය, කඳු නැගීම සහ දිය ඇලි නැරඹීම සඳහා ජනප්‍රිය සංචාරක මධ්‍යස්ථානයකි.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>හෝර්ටන් තැන්න</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>නුවරඑළිය</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>රු. 200 (දේශීය)</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>ලෝකාන්තය සහ බේකර්ස් ඇල්ල පිහිටා ඇති, ජෛව විවිධත්වයෙන් අනූන සුන්දර භූමියකි.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>ශ්‍රී පාදස්ථානය</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>රත්නපුර / නුවරඑළිය</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>නොමිලේ</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>සමනල කන්ද මුදුනේ පිහිටි බෞද්ධ පූජනීය ස්ථානය සහ සුන්දර හිරු උදාවක් දැකිය හැකි ස්ථානයකි.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>මිරිස්ස වෙරළ</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>මාතර</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>නොමිලේ</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>තල්මසුන් නැරඹීම සහ සර්ෆිං (Surfing) ක්‍රීඩාව සඳහා ප්‍රසිද්ධ දකුණු වෙරළ තීරයේ පිහිටි සුන්දර වෙරළකි.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>පින්නවල අලි අනාථාගාරය</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>කෑගල්ල</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>රු. 100 (දේශීය)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>අනාථ වූ අලි ඇතුන් රැකබලා ගන්නා ලොව විශාලතම අලි අනාථාගාරයකි.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>අනුරාධපුර පූජා නගරය</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>අනුරාධපුරය</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>නොමිලේ</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>ශ්‍රී මහා බෝධිය සහ රුවන්වැලිසාය ඇතුළු පැරණි ස්තූප සහිත ඓතිහාසික නගරයකි.</t>
         </is>
       </c>
     </row>

</xml_diff>